<commit_message>
Update FWI forecast and geographic report
</commit_message>
<xml_diff>
--- a/data/FARS_FWI_GeoReport.xlsx
+++ b/data/FARS_FWI_GeoReport.xlsx
@@ -46,99 +46,99 @@
     <t>طبقه خطر</t>
   </si>
   <si>
+    <t>پناهگاه حيات وحش دره باغ</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع توت سياه</t>
+  </si>
+  <si>
+    <t>پارک ملي قطرويه</t>
+  </si>
+  <si>
+    <t>منطقه حفاظت شده بهرام گور</t>
+  </si>
+  <si>
     <t>منطقه شکار ممنوع دره باغ</t>
   </si>
   <si>
-    <t>پناهگاه حيات وحش دره باغ</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع توت سياه</t>
+    <t>منطقه حفاظت شده تنگ سرخ و کوه قلات</t>
   </si>
   <si>
     <t>منطقه شکار ممنوع مل بلند</t>
   </si>
   <si>
-    <t>پارک ملي قطرويه</t>
-  </si>
-  <si>
-    <t>منطقه حفاظت شده بهرام گور</t>
+    <t>منطقه حفاظت شده میانجنگل فسا</t>
+  </si>
+  <si>
+    <t>منطقه حفاظت شده تنگ بستانک</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع کوه دراء</t>
+  </si>
+  <si>
+    <t>پارک ملي بختگان</t>
+  </si>
+  <si>
+    <t>پناهگاه حيات وحش بختگان</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع کوه خم</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع مزايجان</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع روشن کوه</t>
+  </si>
+  <si>
+    <t>منطقه حفاظت شده برم فیروز</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع خرمنکوه</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع کوهستان</t>
   </si>
   <si>
     <t>منطقه شکار ممنوع بصيران</t>
   </si>
   <si>
-    <t>منطقه حفاظت شده تنگ سرخ و کوه قلات</t>
-  </si>
-  <si>
-    <t>منطقه حفاظت شده میانجنگل فسا</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع کوه خم</t>
-  </si>
-  <si>
-    <t>منطقه حفاظت شده برم فیروز</t>
-  </si>
-  <si>
-    <t>منطقه حفاظت شده تنگ بستانک</t>
-  </si>
-  <si>
-    <t>پارک ملي بختگان</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع کوهستان</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع خرمنکوه</t>
-  </si>
-  <si>
-    <t>پناهگاه حيات وحش بختگان</t>
+    <t>منطقه شکار ممنوع کوه گورم</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع دالان</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع بناب</t>
   </si>
   <si>
     <t>پارک ملی بمو</t>
   </si>
   <si>
+    <t>منطقه حفاظت شده ارژن و پريشان</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع کوه سياه</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع کوه خرسي</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع پادنا</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممن.ع آق جلو</t>
+  </si>
+  <si>
+    <t>منطقه شکار ممنوع مهارلو</t>
+  </si>
+  <si>
     <t>منطقه شکار ممنوع شیکوه</t>
   </si>
   <si>
-    <t>منطقه شکار ممنوع کوه گورم</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع کوه دراء</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع کوه خرسي</t>
-  </si>
-  <si>
     <t>منطقه حفاظت شده ماله گاله</t>
   </si>
   <si>
-    <t>منطقه شکار ممنوع بناب</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممن.ع آق جلو</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع کوه سياه</t>
-  </si>
-  <si>
-    <t>منطقه حفاظت شده ارژن و پريشان</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع پادنا</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع روشن کوه</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع مزايجان</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع دالان</t>
-  </si>
-  <si>
-    <t>منطقه شکار ممنوع مهارلو</t>
-  </si>
-  <si>
     <t>منطقه شکار ممنوع کوه هوا و</t>
   </si>
   <si>
@@ -151,16 +151,16 @@
     <t>منطقه حفاظت شده مارگون</t>
   </si>
   <si>
+    <t>مناطق ممنوعه شکار</t>
+  </si>
+  <si>
     <t>مناطق حفاظت‌شده</t>
   </si>
   <si>
-    <t>مناطق ممنوعه شکار</t>
-  </si>
-  <si>
-    <t>1405-06-22</t>
-  </si>
-  <si>
-    <t>2026-09-13</t>
+    <t>1405-06-23</t>
+  </si>
+  <si>
+    <t>2026-09-14</t>
   </si>
   <si>
     <t>بسیار شدید</t>
@@ -628,16 +628,16 @@
         <v>47</v>
       </c>
       <c r="E2">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F2">
-        <v>87.98999999999999</v>
+        <v>89.94</v>
       </c>
       <c r="G2">
-        <v>100.43</v>
+        <v>96.73999999999999</v>
       </c>
       <c r="H2">
-        <v>110.04</v>
+        <v>103.84</v>
       </c>
       <c r="I2" t="s">
         <v>48</v>
@@ -657,16 +657,16 @@
         <v>47</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F3">
-        <v>93.86</v>
+        <v>91.04000000000001</v>
       </c>
       <c r="G3">
-        <v>100</v>
+        <v>94.45</v>
       </c>
       <c r="H3">
-        <v>103.5</v>
+        <v>97.3</v>
       </c>
       <c r="I3" t="s">
         <v>48</v>
@@ -689,13 +689,13 @@
         <v>4</v>
       </c>
       <c r="F4">
-        <v>89.62</v>
+        <v>92.81999999999999</v>
       </c>
       <c r="G4">
-        <v>92.44</v>
+        <v>92.81999999999999</v>
       </c>
       <c r="H4">
-        <v>93.68000000000001</v>
+        <v>92.81999999999999</v>
       </c>
       <c r="I4" t="s">
         <v>48</v>
@@ -715,16 +715,16 @@
         <v>47</v>
       </c>
       <c r="E5">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="F5">
-        <v>81.02</v>
+        <v>84.04000000000001</v>
       </c>
       <c r="G5">
-        <v>89.79000000000001</v>
+        <v>91.18000000000001</v>
       </c>
       <c r="H5">
-        <v>93.66</v>
+        <v>97.18000000000001</v>
       </c>
       <c r="I5" t="s">
         <v>48</v>
@@ -744,16 +744,16 @@
         <v>47</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F6">
-        <v>88.15000000000001</v>
+        <v>67.28</v>
       </c>
       <c r="G6">
-        <v>88.15000000000001</v>
+        <v>89.14</v>
       </c>
       <c r="H6">
-        <v>88.15000000000001</v>
+        <v>103.84</v>
       </c>
       <c r="I6" t="s">
         <v>48</v>
@@ -764,7 +764,7 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
         <v>46</v>
@@ -773,16 +773,16 @@
         <v>47</v>
       </c>
       <c r="E7">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="F7">
-        <v>80.31</v>
+        <v>81.72</v>
       </c>
       <c r="G7">
-        <v>88.11</v>
+        <v>84.48</v>
       </c>
       <c r="H7">
-        <v>93.8</v>
+        <v>88.08</v>
       </c>
       <c r="I7" t="s">
         <v>48</v>
@@ -793,7 +793,7 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C8" t="s">
         <v>46</v>
@@ -802,16 +802,16 @@
         <v>47</v>
       </c>
       <c r="E8">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="F8">
-        <v>57.88</v>
+        <v>75.42</v>
       </c>
       <c r="G8">
-        <v>87.33</v>
+        <v>84.31999999999999</v>
       </c>
       <c r="H8">
-        <v>106.66</v>
+        <v>89.09</v>
       </c>
       <c r="I8" t="s">
         <v>48</v>
@@ -822,7 +822,7 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C9" t="s">
         <v>46</v>
@@ -831,16 +831,16 @@
         <v>47</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="F9">
-        <v>79.98999999999999</v>
+        <v>76.27</v>
       </c>
       <c r="G9">
-        <v>82.76000000000001</v>
+        <v>81.5</v>
       </c>
       <c r="H9">
-        <v>84.92</v>
+        <v>88.78</v>
       </c>
       <c r="I9" t="s">
         <v>48</v>
@@ -851,7 +851,7 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C10" t="s">
         <v>46</v>
@@ -860,16 +860,16 @@
         <v>47</v>
       </c>
       <c r="E10">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="F10">
-        <v>72.64</v>
+        <v>77.36</v>
       </c>
       <c r="G10">
-        <v>79.23999999999999</v>
+        <v>80.73</v>
       </c>
       <c r="H10">
-        <v>88.19</v>
+        <v>85.06</v>
       </c>
       <c r="I10" t="s">
         <v>48</v>
@@ -880,7 +880,7 @@
         <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
         <v>46</v>
@@ -889,16 +889,16 @@
         <v>47</v>
       </c>
       <c r="E11">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="F11">
-        <v>73.44</v>
+        <v>75.13</v>
       </c>
       <c r="G11">
-        <v>78.31</v>
+        <v>80.09</v>
       </c>
       <c r="H11">
-        <v>85.14</v>
+        <v>88.12</v>
       </c>
       <c r="I11" t="s">
         <v>48</v>
@@ -909,7 +909,7 @@
         <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
         <v>46</v>
@@ -918,16 +918,16 @@
         <v>47</v>
       </c>
       <c r="E12">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="F12">
-        <v>72.54000000000001</v>
+        <v>64.93000000000001</v>
       </c>
       <c r="G12">
-        <v>77.92</v>
+        <v>79.86</v>
       </c>
       <c r="H12">
-        <v>83.29000000000001</v>
+        <v>97.61</v>
       </c>
       <c r="I12" t="s">
         <v>48</v>
@@ -938,7 +938,7 @@
         <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
         <v>46</v>
@@ -947,16 +947,16 @@
         <v>47</v>
       </c>
       <c r="E13">
-        <v>5</v>
+        <v>117</v>
       </c>
       <c r="F13">
-        <v>72.03</v>
+        <v>64.93000000000001</v>
       </c>
       <c r="G13">
-        <v>77.5</v>
+        <v>79.23</v>
       </c>
       <c r="H13">
-        <v>80.26000000000001</v>
+        <v>97.61</v>
       </c>
       <c r="I13" t="s">
         <v>48</v>
@@ -976,16 +976,16 @@
         <v>47</v>
       </c>
       <c r="E14">
-        <v>62</v>
+        <v>18</v>
       </c>
       <c r="F14">
-        <v>65.11</v>
+        <v>72.16</v>
       </c>
       <c r="G14">
-        <v>77.03</v>
+        <v>78.89</v>
       </c>
       <c r="H14">
-        <v>97.58</v>
+        <v>85.34999999999999</v>
       </c>
       <c r="I14" t="s">
         <v>48</v>
@@ -996,7 +996,7 @@
         <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C15" t="s">
         <v>46</v>
@@ -1005,16 +1005,16 @@
         <v>47</v>
       </c>
       <c r="E15">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F15">
-        <v>76.64</v>
+        <v>70.56999999999999</v>
       </c>
       <c r="G15">
-        <v>76.64</v>
+        <v>78.7</v>
       </c>
       <c r="H15">
-        <v>76.64</v>
+        <v>83.91</v>
       </c>
       <c r="I15" t="s">
         <v>48</v>
@@ -1025,7 +1025,7 @@
         <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
         <v>46</v>
@@ -1037,13 +1037,13 @@
         <v>12</v>
       </c>
       <c r="F16">
-        <v>72.83</v>
+        <v>74.08</v>
       </c>
       <c r="G16">
-        <v>76.31</v>
+        <v>77.8</v>
       </c>
       <c r="H16">
-        <v>82.67</v>
+        <v>83.2</v>
       </c>
       <c r="I16" t="s">
         <v>48</v>
@@ -1054,7 +1054,7 @@
         <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
         <v>46</v>
@@ -1063,16 +1063,16 @@
         <v>47</v>
       </c>
       <c r="E17">
-        <v>112</v>
+        <v>8</v>
       </c>
       <c r="F17">
-        <v>62.55</v>
+        <v>72.02</v>
       </c>
       <c r="G17">
-        <v>76.22</v>
+        <v>77.61</v>
       </c>
       <c r="H17">
-        <v>97.58</v>
+        <v>82.88</v>
       </c>
       <c r="I17" t="s">
         <v>48</v>
@@ -1092,16 +1092,16 @@
         <v>47</v>
       </c>
       <c r="E18">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F18">
-        <v>66.59</v>
+        <v>74.76000000000001</v>
       </c>
       <c r="G18">
-        <v>75.93000000000001</v>
+        <v>77.56999999999999</v>
       </c>
       <c r="H18">
-        <v>86.64</v>
+        <v>82.83</v>
       </c>
       <c r="I18" t="s">
         <v>48</v>
@@ -1112,7 +1112,7 @@
         <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C19" t="s">
         <v>46</v>
@@ -1121,16 +1121,16 @@
         <v>47</v>
       </c>
       <c r="E19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19">
-        <v>57.45</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="G19">
-        <v>75.91</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="H19">
-        <v>87.26000000000001</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="I19" t="s">
         <v>48</v>
@@ -1141,7 +1141,7 @@
         <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C20" t="s">
         <v>46</v>
@@ -1150,16 +1150,16 @@
         <v>47</v>
       </c>
       <c r="E20">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F20">
-        <v>67.22</v>
+        <v>66.33</v>
       </c>
       <c r="G20">
-        <v>74.91</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="H20">
-        <v>79.97</v>
+        <v>94.58</v>
       </c>
       <c r="I20" t="s">
         <v>48</v>
@@ -1170,7 +1170,7 @@
         <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C21" t="s">
         <v>46</v>
@@ -1179,16 +1179,16 @@
         <v>47</v>
       </c>
       <c r="E21">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="F21">
-        <v>70.13</v>
+        <v>70.94</v>
       </c>
       <c r="G21">
-        <v>74.73</v>
+        <v>76.22</v>
       </c>
       <c r="H21">
-        <v>82</v>
+        <v>80.75</v>
       </c>
       <c r="I21" t="s">
         <v>48</v>
@@ -1199,7 +1199,7 @@
         <v>29</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C22" t="s">
         <v>46</v>
@@ -1208,16 +1208,16 @@
         <v>47</v>
       </c>
       <c r="E22">
-        <v>62</v>
+        <v>8</v>
       </c>
       <c r="F22">
-        <v>67.95</v>
+        <v>74.04000000000001</v>
       </c>
       <c r="G22">
-        <v>73.88</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="H22">
-        <v>83.95</v>
+        <v>77.44</v>
       </c>
       <c r="I22" t="s">
         <v>48</v>
@@ -1237,16 +1237,16 @@
         <v>47</v>
       </c>
       <c r="E23">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F23">
-        <v>70.09</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="G23">
-        <v>73.27</v>
+        <v>75.87</v>
       </c>
       <c r="H23">
-        <v>77.05</v>
+        <v>84.67</v>
       </c>
       <c r="I23" t="s">
         <v>48</v>
@@ -1266,16 +1266,16 @@
         <v>47</v>
       </c>
       <c r="E24">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F24">
-        <v>63.46</v>
+        <v>64.73999999999999</v>
       </c>
       <c r="G24">
-        <v>72.68000000000001</v>
+        <v>75.08</v>
       </c>
       <c r="H24">
-        <v>82.36</v>
+        <v>83.11</v>
       </c>
       <c r="I24" t="s">
         <v>48</v>
@@ -1295,16 +1295,16 @@
         <v>47</v>
       </c>
       <c r="E25">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="F25">
-        <v>71.45</v>
+        <v>67.94</v>
       </c>
       <c r="G25">
-        <v>72.54000000000001</v>
+        <v>73.66</v>
       </c>
       <c r="H25">
-        <v>73.62</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="I25" t="s">
         <v>48</v>
@@ -1315,7 +1315,7 @@
         <v>33</v>
       </c>
       <c r="B26" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C26" t="s">
         <v>46</v>
@@ -1327,13 +1327,13 @@
         <v>13</v>
       </c>
       <c r="F26">
-        <v>69.48999999999999</v>
+        <v>70.12</v>
       </c>
       <c r="G26">
-        <v>72.53</v>
+        <v>73.06999999999999</v>
       </c>
       <c r="H26">
-        <v>74.93000000000001</v>
+        <v>78.17</v>
       </c>
       <c r="I26" t="s">
         <v>48</v>
@@ -1353,16 +1353,16 @@
         <v>47</v>
       </c>
       <c r="E27">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="F27">
-        <v>64.08</v>
+        <v>64.20999999999999</v>
       </c>
       <c r="G27">
-        <v>72.36</v>
+        <v>72.81</v>
       </c>
       <c r="H27">
-        <v>75.58</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="I27" t="s">
         <v>48</v>
@@ -1373,7 +1373,7 @@
         <v>35</v>
       </c>
       <c r="B28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C28" t="s">
         <v>46</v>
@@ -1385,13 +1385,13 @@
         <v>20</v>
       </c>
       <c r="F28">
-        <v>65.14</v>
+        <v>65</v>
       </c>
       <c r="G28">
-        <v>71.93000000000001</v>
+        <v>72.73999999999999</v>
       </c>
       <c r="H28">
-        <v>82.09</v>
+        <v>84.39</v>
       </c>
       <c r="I28" t="s">
         <v>48</v>
@@ -1402,7 +1402,7 @@
         <v>36</v>
       </c>
       <c r="B29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C29" t="s">
         <v>46</v>
@@ -1411,16 +1411,16 @@
         <v>47</v>
       </c>
       <c r="E29">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F29">
-        <v>64.83</v>
+        <v>69.61</v>
       </c>
       <c r="G29">
-        <v>71.64</v>
+        <v>72.37</v>
       </c>
       <c r="H29">
-        <v>78.48</v>
+        <v>75.14</v>
       </c>
       <c r="I29" t="s">
         <v>48</v>
@@ -1431,7 +1431,7 @@
         <v>37</v>
       </c>
       <c r="B30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C30" t="s">
         <v>46</v>
@@ -1440,16 +1440,16 @@
         <v>47</v>
       </c>
       <c r="E30">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F30">
-        <v>66.58</v>
+        <v>61.31</v>
       </c>
       <c r="G30">
         <v>70.91</v>
       </c>
       <c r="H30">
-        <v>76.23</v>
+        <v>77.84</v>
       </c>
       <c r="I30" t="s">
         <v>48</v>
@@ -1460,7 +1460,7 @@
         <v>38</v>
       </c>
       <c r="B31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C31" t="s">
         <v>46</v>
@@ -1469,19 +1469,19 @@
         <v>47</v>
       </c>
       <c r="E31">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F31">
-        <v>67.91</v>
+        <v>65.98</v>
       </c>
       <c r="G31">
-        <v>69.81999999999999</v>
+        <v>70.83</v>
       </c>
       <c r="H31">
-        <v>71.43000000000001</v>
+        <v>73.39</v>
       </c>
       <c r="I31" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -1498,16 +1498,16 @@
         <v>47</v>
       </c>
       <c r="E32">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F32">
-        <v>61.23</v>
+        <v>65.09</v>
       </c>
       <c r="G32">
-        <v>67.09</v>
+        <v>69.42</v>
       </c>
       <c r="H32">
-        <v>72.62</v>
+        <v>74.89</v>
       </c>
       <c r="I32" t="s">
         <v>49</v>
@@ -1518,7 +1518,7 @@
         <v>40</v>
       </c>
       <c r="B33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C33" t="s">
         <v>46</v>
@@ -1530,13 +1530,13 @@
         <v>37</v>
       </c>
       <c r="F33">
-        <v>55.11</v>
+        <v>55.18</v>
       </c>
       <c r="G33">
-        <v>62.76</v>
+        <v>64.42</v>
       </c>
       <c r="H33">
-        <v>74.62</v>
+        <v>78.63</v>
       </c>
       <c r="I33" t="s">
         <v>49</v>
@@ -1547,7 +1547,7 @@
         <v>41</v>
       </c>
       <c r="B34" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C34" t="s">
         <v>46</v>
@@ -1559,13 +1559,13 @@
         <v>9</v>
       </c>
       <c r="F34">
-        <v>51.79</v>
+        <v>52.46</v>
       </c>
       <c r="G34">
-        <v>57.6</v>
+        <v>56.83</v>
       </c>
       <c r="H34">
-        <v>62.94</v>
+        <v>64.94</v>
       </c>
       <c r="I34" t="s">
         <v>49</v>
@@ -1576,7 +1576,7 @@
         <v>42</v>
       </c>
       <c r="B35" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C35" t="s">
         <v>46</v>
@@ -1596,7 +1596,7 @@
         <v>43</v>
       </c>
       <c r="B36" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C36" t="s">
         <v>46</v>

</xml_diff>